<commit_message>
cal_error() based on grant-assisted B2s
</commit_message>
<xml_diff>
--- a/inst/extdata/scenario_parameters.xlsx
+++ b/inst/extdata/scenario_parameters.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Joe\pkgs\hpmicrosimr\inst\extdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E0BF7B19-603C-4C9A-961C-3BA34090B5B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2713132B-FA25-40AB-A297-CF99FD718ED5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Description" sheetId="7" r:id="rId1"/>
@@ -18,6 +18,8 @@
     <sheet name="WAM" sheetId="17" r:id="rId3"/>
     <sheet name="CAP" sheetId="19" r:id="rId4"/>
     <sheet name="DWIT" sheetId="18" r:id="rId5"/>
+    <sheet name="HighSpark" sheetId="20" r:id="rId6"/>
+    <sheet name="LowSpark" sheetId="21" r:id="rId7"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -40,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1377" uniqueCount="234">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2057" uniqueCount="238">
   <si>
     <t>category</t>
   </si>
@@ -726,29 +728,71 @@
     <t>ireland 2000-2020 IEA 2196, included effect of solar gain</t>
   </si>
   <si>
-    <t>LowSparkGap</t>
-  </si>
-  <si>
-    <t>Same as WAM but Spark Gap falls</t>
-  </si>
-  <si>
-    <t>HighSparkGap</t>
-  </si>
-  <si>
-    <t>Same as WAM but Spark Gap rises</t>
-  </si>
-  <si>
     <t>oil prices excluding carbon tax</t>
   </si>
   <si>
     <t>gas prices excluding carbon tax</t>
+  </si>
+  <si>
+    <t>HighSpark</t>
+  </si>
+  <si>
+    <t>LowSpark</t>
+  </si>
+  <si>
+    <t>"High Spark Gap"</t>
+  </si>
+  <si>
+    <t>"Low spark gap"</t>
+  </si>
+  <si>
+    <t>high network costs</t>
+  </si>
+  <si>
+    <t>same as CAP but with high CT assumption</t>
+  </si>
+  <si>
+    <t>same as CAP but CT frozen at 100 and higher electricity prices</t>
+  </si>
+  <si>
+    <r>
+      <t>(1) carbon tax increases to 100 in 2030 but stays flat at this level (2) electricity price increases to 0.45</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>€</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>/kWh in 2040,driven by higher network costs</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -784,6 +828,18 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="8">
@@ -874,7 +930,7 @@
     <xf numFmtId="0" fontId="3" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="3" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -904,6 +960,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="7">
@@ -1310,20 +1369,29 @@
         <v>214</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A7" s="2" t="s">
-        <v>228</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>229</v>
+    <row r="7" spans="1:4" s="22" customFormat="1" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A7" s="22" t="s">
+        <v>230</v>
+      </c>
+      <c r="B7" s="22" t="s">
+        <v>232</v>
+      </c>
+      <c r="C7" s="22" t="s">
+        <v>236</v>
+      </c>
+      <c r="D7" s="22" t="s">
+        <v>237</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>231</v>
+        <v>233</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>235</v>
       </c>
     </row>
   </sheetData>
@@ -1852,7 +1920,7 @@
         <v>43</v>
       </c>
       <c r="B29" s="5" t="s">
-        <v>232</v>
+        <v>228</v>
       </c>
       <c r="C29" s="5" t="s">
         <v>45</v>
@@ -1904,7 +1972,7 @@
         <v>43</v>
       </c>
       <c r="B32" s="5" t="s">
-        <v>233</v>
+        <v>229</v>
       </c>
       <c r="C32" s="5" t="s">
         <v>224</v>
@@ -2050,7 +2118,7 @@
         <v>93</v>
       </c>
       <c r="D40" s="5">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="E40" s="5"/>
     </row>
@@ -2065,7 +2133,7 @@
         <v>94</v>
       </c>
       <c r="D41" s="5">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="E41" s="5"/>
     </row>
@@ -2080,7 +2148,7 @@
         <v>95</v>
       </c>
       <c r="D42" s="5">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="E42" s="5"/>
     </row>
@@ -2095,7 +2163,7 @@
         <v>96</v>
       </c>
       <c r="D43" s="5">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="E43" s="5"/>
     </row>
@@ -2266,7 +2334,7 @@
         <v>124</v>
       </c>
       <c r="D54" s="13">
-        <v>150</v>
+        <v>120</v>
       </c>
       <c r="E54" s="13" t="s">
         <v>102</v>
@@ -3530,7 +3598,7 @@
         <v>93</v>
       </c>
       <c r="D40" s="5">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="E40" s="5"/>
     </row>
@@ -3545,7 +3613,7 @@
         <v>94</v>
       </c>
       <c r="D41" s="5">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="E41" s="5"/>
     </row>
@@ -3560,7 +3628,7 @@
         <v>95</v>
       </c>
       <c r="D42" s="5">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="E42" s="5"/>
     </row>
@@ -3575,7 +3643,7 @@
         <v>96</v>
       </c>
       <c r="D43" s="5">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="E43" s="5"/>
     </row>
@@ -5010,7 +5078,7 @@
         <v>93</v>
       </c>
       <c r="D40" s="5">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="E40" s="5"/>
     </row>
@@ -5025,7 +5093,7 @@
         <v>94</v>
       </c>
       <c r="D41" s="5">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="E41" s="5"/>
     </row>
@@ -5040,7 +5108,7 @@
         <v>95</v>
       </c>
       <c r="D42" s="5">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="E42" s="5"/>
     </row>
@@ -5055,7 +5123,7 @@
         <v>96</v>
       </c>
       <c r="D43" s="5">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="E43" s="5"/>
     </row>
@@ -6490,7 +6558,7 @@
         <v>93</v>
       </c>
       <c r="D40" s="5">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="E40" s="5"/>
       <c r="F40" s="5"/>
@@ -6506,7 +6574,7 @@
         <v>94</v>
       </c>
       <c r="D41" s="5">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="E41" s="5"/>
     </row>
@@ -6521,7 +6589,7 @@
         <v>95</v>
       </c>
       <c r="D42" s="5">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="E42" s="5"/>
     </row>
@@ -6536,7 +6604,7 @@
         <v>96</v>
       </c>
       <c r="D43" s="5">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="E43" s="5"/>
     </row>
@@ -7029,6 +7097,2969 @@
       </c>
       <c r="D74" s="13">
         <v>3</v>
+      </c>
+    </row>
+    <row r="75" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A75" s="11" t="s">
+        <v>6</v>
+      </c>
+      <c r="B75" s="13" t="s">
+        <v>201</v>
+      </c>
+      <c r="C75" s="13" t="s">
+        <v>202</v>
+      </c>
+      <c r="D75" s="13">
+        <v>2035</v>
+      </c>
+    </row>
+    <row r="76" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A76" s="17" t="s">
+        <v>114</v>
+      </c>
+      <c r="B76" s="18" t="s">
+        <v>115</v>
+      </c>
+      <c r="C76" s="18" t="s">
+        <v>113</v>
+      </c>
+      <c r="D76" s="18">
+        <v>3000</v>
+      </c>
+      <c r="E76" t="s">
+        <v>22</v>
+      </c>
+      <c r="F76" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="77" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A77" s="17" t="s">
+        <v>114</v>
+      </c>
+      <c r="B77" s="18" t="s">
+        <v>116</v>
+      </c>
+      <c r="C77" s="18" t="s">
+        <v>117</v>
+      </c>
+      <c r="D77" s="18">
+        <v>75</v>
+      </c>
+      <c r="E77" t="s">
+        <v>102</v>
+      </c>
+      <c r="F77" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="78" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A78" t="s">
+        <v>10</v>
+      </c>
+      <c r="B78" t="s">
+        <v>14</v>
+      </c>
+      <c r="C78" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="D78">
+        <v>0.35</v>
+      </c>
+      <c r="E78" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="79" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A79" t="s">
+        <v>10</v>
+      </c>
+      <c r="B79" t="s">
+        <v>16</v>
+      </c>
+      <c r="C79" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="D79">
+        <v>5.68692529674572E-2</v>
+      </c>
+      <c r="E79" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="80" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A80" t="s">
+        <v>10</v>
+      </c>
+      <c r="B80" t="s">
+        <v>15</v>
+      </c>
+      <c r="C80" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="D80" s="3">
+        <v>0</v>
+      </c>
+      <c r="E80" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="81" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A81" t="s">
+        <v>10</v>
+      </c>
+      <c r="B81" t="s">
+        <v>9</v>
+      </c>
+      <c r="C81" s="3" t="s">
+        <v>107</v>
+      </c>
+      <c r="D81">
+        <v>4.2307926455512603E-2</v>
+      </c>
+      <c r="E81" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="82" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A82" t="s">
+        <v>10</v>
+      </c>
+      <c r="B82" t="s">
+        <v>87</v>
+      </c>
+      <c r="C82" s="14" t="s">
+        <v>11</v>
+      </c>
+      <c r="D82">
+        <v>0.57089503190107604</v>
+      </c>
+      <c r="E82" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="83" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A83" t="s">
+        <v>10</v>
+      </c>
+      <c r="B83" t="s">
+        <v>151</v>
+      </c>
+      <c r="C83" s="14" t="s">
+        <v>128</v>
+      </c>
+      <c r="D83">
+        <v>0.102978633031016</v>
+      </c>
+      <c r="E83" t="s">
+        <v>68</v>
+      </c>
+      <c r="F83" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="84" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A84" t="s">
+        <v>10</v>
+      </c>
+      <c r="B84" t="s">
+        <v>106</v>
+      </c>
+      <c r="C84" s="14" t="s">
+        <v>127</v>
+      </c>
+      <c r="D84" s="3">
+        <v>0.4</v>
+      </c>
+      <c r="E84" t="s">
+        <v>68</v>
+      </c>
+      <c r="F84" s="16">
+        <v>0.3</v>
+      </c>
+    </row>
+    <row r="85" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A85" t="s">
+        <v>10</v>
+      </c>
+      <c r="B85" t="s">
+        <v>140</v>
+      </c>
+      <c r="C85" s="14" t="s">
+        <v>141</v>
+      </c>
+      <c r="D85" s="3">
+        <v>0</v>
+      </c>
+      <c r="E85" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="86" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A86" t="s">
+        <v>10</v>
+      </c>
+      <c r="B86" t="s">
+        <v>154</v>
+      </c>
+      <c r="C86" s="14" t="s">
+        <v>152</v>
+      </c>
+      <c r="D86">
+        <v>2.86857836910057E-2</v>
+      </c>
+      <c r="E86" t="s">
+        <v>68</v>
+      </c>
+      <c r="F86" t="s">
+        <v>153</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{39B4A857-0D5A-4339-92CB-200FF0EB3A2A}">
+  <dimension ref="A1:F86"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="25.44140625" customWidth="1"/>
+    <col min="2" max="2" width="30.77734375" customWidth="1"/>
+    <col min="3" max="3" width="32.5546875" customWidth="1"/>
+    <col min="4" max="4" width="24.21875" customWidth="1"/>
+    <col min="5" max="5" width="25.44140625" customWidth="1"/>
+    <col min="6" max="6" width="27.77734375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A2" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="D2" s="4">
+        <v>2000</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="F2" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A3" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="D3" s="4">
+        <v>16</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A4" s="4" t="s">
+        <v>163</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>164</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>165</v>
+      </c>
+      <c r="D4" s="4">
+        <v>2.5000000000000001E-3</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="F4" s="4" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A5" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="B5" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="C5" s="7" t="s">
+        <v>100</v>
+      </c>
+      <c r="D5" s="7">
+        <v>30</v>
+      </c>
+      <c r="E5" s="6" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A6" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="B6" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="C6" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="D6" s="6">
+        <v>40</v>
+      </c>
+      <c r="E6" s="6" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A7" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="B7" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="C7" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="D7" s="7">
+        <v>60</v>
+      </c>
+      <c r="E7" s="7" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A8" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="B8" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="C8" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="D8" s="7">
+        <v>60</v>
+      </c>
+      <c r="E8" s="7" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A9" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="B9" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="C9" s="8" t="s">
+        <v>57</v>
+      </c>
+      <c r="D9" s="8">
+        <v>60</v>
+      </c>
+      <c r="E9" s="8" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A10" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="B10" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="C10" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="D10" s="6">
+        <v>150</v>
+      </c>
+      <c r="E10" s="6" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A11" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="B11" s="7" t="s">
+        <v>64</v>
+      </c>
+      <c r="C11" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="D11" s="7">
+        <v>130</v>
+      </c>
+      <c r="E11" s="7" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A12" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="B12" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="C12" s="7" t="s">
+        <v>62</v>
+      </c>
+      <c r="D12" s="7">
+        <v>200</v>
+      </c>
+      <c r="E12" s="7" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A13" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="B13" s="7" t="s">
+        <v>66</v>
+      </c>
+      <c r="C13" s="7" t="s">
+        <v>63</v>
+      </c>
+      <c r="D13" s="7">
+        <v>70</v>
+      </c>
+      <c r="E13" s="7" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A14" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="B14" s="8" t="s">
+        <v>217</v>
+      </c>
+      <c r="C14" s="8" t="s">
+        <v>218</v>
+      </c>
+      <c r="D14" s="8">
+        <v>120</v>
+      </c>
+      <c r="E14" s="8" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A15" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="B15" s="7" t="s">
+        <v>83</v>
+      </c>
+      <c r="C15" s="7" t="s">
+        <v>82</v>
+      </c>
+      <c r="D15" s="7">
+        <v>110</v>
+      </c>
+      <c r="E15" s="8" t="s">
+        <v>85</v>
+      </c>
+      <c r="F15" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A16" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="B16" s="7" t="s">
+        <v>80</v>
+      </c>
+      <c r="C16" s="7" t="s">
+        <v>81</v>
+      </c>
+      <c r="D16" s="7">
+        <v>0.81</v>
+      </c>
+      <c r="E16" s="7" t="s">
+        <v>68</v>
+      </c>
+      <c r="F16" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A17" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="B17" s="7" t="s">
+        <v>111</v>
+      </c>
+      <c r="C17" s="7" t="s">
+        <v>109</v>
+      </c>
+      <c r="D17" s="7">
+        <v>0</v>
+      </c>
+      <c r="E17" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="F17" s="7" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A18" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="B18" s="7" t="s">
+        <v>119</v>
+      </c>
+      <c r="C18" s="7" t="s">
+        <v>121</v>
+      </c>
+      <c r="D18" s="7">
+        <v>0.3</v>
+      </c>
+      <c r="E18" s="7" t="s">
+        <v>68</v>
+      </c>
+      <c r="F18" s="7" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A19" s="15" t="s">
+        <v>17</v>
+      </c>
+      <c r="B19" s="15" t="s">
+        <v>130</v>
+      </c>
+      <c r="C19" s="15" t="s">
+        <v>101</v>
+      </c>
+      <c r="D19" s="15">
+        <v>30</v>
+      </c>
+      <c r="E19" s="15" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A20" s="15" t="s">
+        <v>17</v>
+      </c>
+      <c r="B20" s="15" t="s">
+        <v>103</v>
+      </c>
+      <c r="C20" s="15" t="s">
+        <v>108</v>
+      </c>
+      <c r="D20" s="15">
+        <v>30</v>
+      </c>
+      <c r="E20" s="15" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A21" s="15" t="s">
+        <v>17</v>
+      </c>
+      <c r="B21" s="15" t="s">
+        <v>104</v>
+      </c>
+      <c r="C21" s="15" t="s">
+        <v>105</v>
+      </c>
+      <c r="D21" s="15">
+        <v>8</v>
+      </c>
+      <c r="E21" s="15" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A22" s="15" t="s">
+        <v>17</v>
+      </c>
+      <c r="B22" s="15" t="s">
+        <v>129</v>
+      </c>
+      <c r="C22" s="15" t="s">
+        <v>131</v>
+      </c>
+      <c r="D22" s="15">
+        <v>2.2999999999999998</v>
+      </c>
+      <c r="E22" s="15" t="s">
+        <v>132</v>
+      </c>
+      <c r="F22" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A23" s="15" t="s">
+        <v>17</v>
+      </c>
+      <c r="B23" s="15" t="s">
+        <v>134</v>
+      </c>
+      <c r="C23" s="15" t="s">
+        <v>137</v>
+      </c>
+      <c r="D23" s="15">
+        <v>1.25</v>
+      </c>
+      <c r="E23" s="15"/>
+      <c r="F23" s="15" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A24" s="15" t="s">
+        <v>17</v>
+      </c>
+      <c r="B24" s="15" t="s">
+        <v>135</v>
+      </c>
+      <c r="C24" s="15" t="s">
+        <v>138</v>
+      </c>
+      <c r="D24" s="15">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="E24" s="15"/>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A25" s="15" t="s">
+        <v>17</v>
+      </c>
+      <c r="B25" s="15" t="s">
+        <v>136</v>
+      </c>
+      <c r="C25" s="15" t="s">
+        <v>139</v>
+      </c>
+      <c r="D25" s="15">
+        <v>1.08</v>
+      </c>
+      <c r="E25" s="15"/>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A26" s="15" t="s">
+        <v>17</v>
+      </c>
+      <c r="B26" s="15" t="s">
+        <v>179</v>
+      </c>
+      <c r="C26" s="15" t="s">
+        <v>180</v>
+      </c>
+      <c r="D26" s="15">
+        <v>0.3</v>
+      </c>
+      <c r="E26" s="15" t="s">
+        <v>68</v>
+      </c>
+      <c r="F26" s="15" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A27" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="B27" s="10" t="s">
+        <v>99</v>
+      </c>
+      <c r="C27" s="10" t="s">
+        <v>181</v>
+      </c>
+      <c r="D27" s="10">
+        <v>0.6</v>
+      </c>
+      <c r="E27" s="10" t="s">
+        <v>68</v>
+      </c>
+      <c r="F27" s="9" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A28" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="B28" s="5" t="s">
+        <v>69</v>
+      </c>
+      <c r="C28" s="5" t="s">
+        <v>223</v>
+      </c>
+      <c r="D28" s="5">
+        <v>11.8</v>
+      </c>
+      <c r="E28" s="5" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A29" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="B29" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="C29" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="D29" s="5">
+        <v>11.8</v>
+      </c>
+      <c r="E29" s="5" t="s">
+        <v>146</v>
+      </c>
+      <c r="F29" s="5"/>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A30" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="B30" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="C30" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="D30" s="5">
+        <v>11.8</v>
+      </c>
+      <c r="E30" s="5" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A31" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="B31" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="C31" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="D31" s="5">
+        <v>11.8</v>
+      </c>
+      <c r="E31" s="5" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A32" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="B32" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="C32" s="5" t="s">
+        <v>224</v>
+      </c>
+      <c r="D32" s="5">
+        <v>13.2</v>
+      </c>
+      <c r="E32" s="5" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A33" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="B33" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="C33" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="D33" s="5">
+        <v>13.2</v>
+      </c>
+      <c r="E33" s="5" t="s">
+        <v>146</v>
+      </c>
+      <c r="F33" s="5" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A34" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="B34" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="C34" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="D34" s="5">
+        <v>13.2</v>
+      </c>
+      <c r="E34" s="5" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A35" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="B35" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="C35" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="D35" s="5">
+        <v>13.2</v>
+      </c>
+      <c r="E35" s="5" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A36" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="B36" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="C36" s="5" t="s">
+        <v>225</v>
+      </c>
+      <c r="D36" s="5">
+        <v>35.4</v>
+      </c>
+      <c r="E36" s="5" t="s">
+        <v>146</v>
+      </c>
+      <c r="F36" s="5"/>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A37" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="B37" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="C37" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="D37" s="5">
+        <v>40</v>
+      </c>
+      <c r="E37" s="5" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A38" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="B38" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="C38" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="D38" s="5">
+        <v>42</v>
+      </c>
+      <c r="E38" s="5" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A39" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="B39" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="C39" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D39" s="5">
+        <v>45</v>
+      </c>
+      <c r="E39" s="5" t="s">
+        <v>146</v>
+      </c>
+      <c r="F39" s="5" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A40" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="B40" s="5" t="s">
+        <v>90</v>
+      </c>
+      <c r="C40" s="5" t="s">
+        <v>93</v>
+      </c>
+      <c r="D40" s="5">
+        <v>0.3</v>
+      </c>
+      <c r="E40" s="5"/>
+      <c r="F40" s="5"/>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A41" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="B41" s="5" t="s">
+        <v>90</v>
+      </c>
+      <c r="C41" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="D41" s="5">
+        <v>0.3</v>
+      </c>
+      <c r="E41" s="5"/>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A42" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="B42" s="5" t="s">
+        <v>90</v>
+      </c>
+      <c r="C42" s="5" t="s">
+        <v>95</v>
+      </c>
+      <c r="D42" s="5">
+        <v>0.3</v>
+      </c>
+      <c r="E42" s="5"/>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A43" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="B43" s="5" t="s">
+        <v>90</v>
+      </c>
+      <c r="C43" s="5" t="s">
+        <v>96</v>
+      </c>
+      <c r="D43" s="5">
+        <v>0.3</v>
+      </c>
+      <c r="E43" s="5"/>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A44" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="B44" s="5" t="s">
+        <v>222</v>
+      </c>
+      <c r="C44" s="5" t="s">
+        <v>226</v>
+      </c>
+      <c r="D44" s="5">
+        <v>11.4</v>
+      </c>
+      <c r="E44" s="5"/>
+      <c r="F44" s="5" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A45" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="B45" s="5" t="s">
+        <v>222</v>
+      </c>
+      <c r="C45" s="5" t="s">
+        <v>219</v>
+      </c>
+      <c r="D45" s="5">
+        <v>11.4</v>
+      </c>
+      <c r="E45" s="5"/>
+      <c r="F45" s="5" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A46" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="B46" s="5" t="s">
+        <v>222</v>
+      </c>
+      <c r="C46" s="5" t="s">
+        <v>220</v>
+      </c>
+      <c r="D46" s="5">
+        <v>11.4</v>
+      </c>
+      <c r="E46" s="5"/>
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A47" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="B47" s="5" t="s">
+        <v>222</v>
+      </c>
+      <c r="C47" s="5" t="s">
+        <v>221</v>
+      </c>
+      <c r="D47" s="5">
+        <v>11.4</v>
+      </c>
+      <c r="E47" s="5"/>
+    </row>
+    <row r="48" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A48" s="11" t="s">
+        <v>6</v>
+      </c>
+      <c r="B48" s="11" t="s">
+        <v>174</v>
+      </c>
+      <c r="C48" s="12" t="s">
+        <v>175</v>
+      </c>
+      <c r="D48" s="13">
+        <v>700</v>
+      </c>
+      <c r="E48" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A49" s="11" t="s">
+        <v>6</v>
+      </c>
+      <c r="B49" s="11" t="s">
+        <v>39</v>
+      </c>
+      <c r="C49" s="12" t="s">
+        <v>41</v>
+      </c>
+      <c r="D49" s="13">
+        <v>0.13500000000000001</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A50" s="11" t="s">
+        <v>6</v>
+      </c>
+      <c r="B50" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="C50" s="12" t="s">
+        <v>42</v>
+      </c>
+      <c r="D50" s="13">
+        <v>0.23</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A51" s="11" t="s">
+        <v>6</v>
+      </c>
+      <c r="B51" s="13" t="s">
+        <v>70</v>
+      </c>
+      <c r="C51" s="12" t="s">
+        <v>76</v>
+      </c>
+      <c r="D51" s="13">
+        <v>2018.3</v>
+      </c>
+      <c r="E51" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A52" s="11" t="s">
+        <v>6</v>
+      </c>
+      <c r="B52" s="13" t="s">
+        <v>71</v>
+      </c>
+      <c r="C52" s="12" t="s">
+        <v>78</v>
+      </c>
+      <c r="D52" s="13">
+        <v>2022.15</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A53" s="11" t="s">
+        <v>6</v>
+      </c>
+      <c r="B53" s="13" t="s">
+        <v>88</v>
+      </c>
+      <c r="C53" s="12" t="s">
+        <v>89</v>
+      </c>
+      <c r="D53" s="13">
+        <v>2011</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A54" s="11" t="s">
+        <v>6</v>
+      </c>
+      <c r="B54" s="13" t="s">
+        <v>122</v>
+      </c>
+      <c r="C54" s="12" t="s">
+        <v>124</v>
+      </c>
+      <c r="D54" s="13">
+        <v>150</v>
+      </c>
+      <c r="E54" s="13" t="s">
+        <v>102</v>
+      </c>
+      <c r="F54" s="13" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A55" s="11" t="s">
+        <v>6</v>
+      </c>
+      <c r="B55" s="13" t="s">
+        <v>176</v>
+      </c>
+      <c r="C55" s="12" t="s">
+        <v>178</v>
+      </c>
+      <c r="D55" s="13">
+        <v>35000</v>
+      </c>
+      <c r="E55" s="13" t="s">
+        <v>22</v>
+      </c>
+      <c r="F55" s="13"/>
+    </row>
+    <row r="56" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A56" s="11" t="s">
+        <v>6</v>
+      </c>
+      <c r="B56" s="13" t="s">
+        <v>123</v>
+      </c>
+      <c r="C56" s="12" t="s">
+        <v>125</v>
+      </c>
+      <c r="D56" s="13">
+        <v>2027</v>
+      </c>
+      <c r="E56" s="13" t="s">
+        <v>126</v>
+      </c>
+      <c r="F56" s="13" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="57" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A57" s="11" t="s">
+        <v>6</v>
+      </c>
+      <c r="B57" s="13" t="s">
+        <v>203</v>
+      </c>
+      <c r="C57" s="12" t="s">
+        <v>205</v>
+      </c>
+      <c r="D57" s="13">
+        <v>2028</v>
+      </c>
+      <c r="E57" s="13"/>
+      <c r="F57" s="13"/>
+    </row>
+    <row r="58" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A58" s="11" t="s">
+        <v>6</v>
+      </c>
+      <c r="B58" s="13" t="s">
+        <v>210</v>
+      </c>
+      <c r="C58" s="12" t="s">
+        <v>209</v>
+      </c>
+      <c r="D58" s="13">
+        <v>100</v>
+      </c>
+      <c r="E58" s="13" t="s">
+        <v>208</v>
+      </c>
+      <c r="F58" s="13"/>
+    </row>
+    <row r="59" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A59" s="11" t="s">
+        <v>6</v>
+      </c>
+      <c r="B59" s="13" t="s">
+        <v>206</v>
+      </c>
+      <c r="C59" s="12" t="s">
+        <v>207</v>
+      </c>
+      <c r="D59" s="13">
+        <v>50000</v>
+      </c>
+      <c r="E59" s="13" t="s">
+        <v>22</v>
+      </c>
+      <c r="F59" s="13"/>
+    </row>
+    <row r="60" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A60" s="11" t="s">
+        <v>6</v>
+      </c>
+      <c r="B60" s="13" t="s">
+        <v>97</v>
+      </c>
+      <c r="C60" s="12" t="s">
+        <v>98</v>
+      </c>
+      <c r="D60" s="13">
+        <v>2015.3</v>
+      </c>
+    </row>
+    <row r="61" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A61" s="11" t="s">
+        <v>6</v>
+      </c>
+      <c r="B61" s="13" t="s">
+        <v>72</v>
+      </c>
+      <c r="C61" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="D61" s="13">
+        <v>2024.3</v>
+      </c>
+      <c r="E61" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A62" s="11" t="s">
+        <v>6</v>
+      </c>
+      <c r="B62" s="13" t="s">
+        <v>79</v>
+      </c>
+      <c r="C62" s="12" t="s">
+        <v>77</v>
+      </c>
+      <c r="D62" s="13">
+        <v>2040</v>
+      </c>
+    </row>
+    <row r="63" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A63" s="11" t="s">
+        <v>6</v>
+      </c>
+      <c r="B63" s="13" t="s">
+        <v>91</v>
+      </c>
+      <c r="C63" s="12" t="s">
+        <v>92</v>
+      </c>
+      <c r="D63" s="13">
+        <v>2040</v>
+      </c>
+    </row>
+    <row r="64" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A64" s="11" t="s">
+        <v>6</v>
+      </c>
+      <c r="B64" s="13" t="s">
+        <v>142</v>
+      </c>
+      <c r="C64" s="13" t="s">
+        <v>144</v>
+      </c>
+      <c r="D64" s="13">
+        <v>0.8</v>
+      </c>
+      <c r="E64" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="65" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A65" s="11" t="s">
+        <v>6</v>
+      </c>
+      <c r="B65" s="13" t="s">
+        <v>197</v>
+      </c>
+      <c r="C65" s="13" t="s">
+        <v>193</v>
+      </c>
+      <c r="D65" s="13">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="66" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A66" s="11" t="s">
+        <v>6</v>
+      </c>
+      <c r="B66" s="13" t="s">
+        <v>170</v>
+      </c>
+      <c r="C66" s="13" t="s">
+        <v>194</v>
+      </c>
+      <c r="D66" s="13">
+        <v>63.5</v>
+      </c>
+      <c r="E66" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A67" s="11" t="s">
+        <v>6</v>
+      </c>
+      <c r="B67" s="13" t="s">
+        <v>171</v>
+      </c>
+      <c r="C67" s="13" t="s">
+        <v>195</v>
+      </c>
+      <c r="D67" s="13">
+        <v>100</v>
+      </c>
+      <c r="E67" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="68" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A68" s="11" t="s">
+        <v>6</v>
+      </c>
+      <c r="B68" s="13" t="s">
+        <v>172</v>
+      </c>
+      <c r="C68" s="13" t="s">
+        <v>196</v>
+      </c>
+      <c r="D68" s="13">
+        <v>100</v>
+      </c>
+      <c r="E68" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="69" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A69" s="11" t="s">
+        <v>6</v>
+      </c>
+      <c r="B69" s="13" t="s">
+        <v>185</v>
+      </c>
+      <c r="C69" s="13" t="s">
+        <v>187</v>
+      </c>
+      <c r="D69" s="13">
+        <v>2026.5</v>
+      </c>
+    </row>
+    <row r="70" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A70" s="11" t="s">
+        <v>6</v>
+      </c>
+      <c r="B70" s="13" t="s">
+        <v>186</v>
+      </c>
+      <c r="C70" s="13" t="s">
+        <v>188</v>
+      </c>
+      <c r="D70" s="13">
+        <v>1.65</v>
+      </c>
+    </row>
+    <row r="71" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A71" s="11" t="s">
+        <v>6</v>
+      </c>
+      <c r="B71" s="13" t="s">
+        <v>190</v>
+      </c>
+      <c r="C71" s="13" t="s">
+        <v>189</v>
+      </c>
+      <c r="D71" s="13">
+        <v>2028</v>
+      </c>
+    </row>
+    <row r="72" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A72" s="11" t="s">
+        <v>6</v>
+      </c>
+      <c r="B72" s="13" t="s">
+        <v>191</v>
+      </c>
+      <c r="C72" s="13" t="s">
+        <v>192</v>
+      </c>
+      <c r="D72" s="13">
+        <v>2041</v>
+      </c>
+    </row>
+    <row r="73" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A73" s="11" t="s">
+        <v>6</v>
+      </c>
+      <c r="B73" s="13" t="s">
+        <v>129</v>
+      </c>
+      <c r="C73" s="13" t="s">
+        <v>198</v>
+      </c>
+      <c r="D73" s="13">
+        <v>2028</v>
+      </c>
+    </row>
+    <row r="74" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A74" s="11" t="s">
+        <v>6</v>
+      </c>
+      <c r="B74" s="13" t="s">
+        <v>129</v>
+      </c>
+      <c r="C74" s="13" t="s">
+        <v>199</v>
+      </c>
+      <c r="D74" s="13">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="75" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A75" s="11" t="s">
+        <v>6</v>
+      </c>
+      <c r="B75" s="13" t="s">
+        <v>201</v>
+      </c>
+      <c r="C75" s="13" t="s">
+        <v>202</v>
+      </c>
+      <c r="D75" s="13">
+        <v>2035</v>
+      </c>
+    </row>
+    <row r="76" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A76" s="17" t="s">
+        <v>114</v>
+      </c>
+      <c r="B76" s="18" t="s">
+        <v>115</v>
+      </c>
+      <c r="C76" s="18" t="s">
+        <v>113</v>
+      </c>
+      <c r="D76" s="18">
+        <v>3000</v>
+      </c>
+      <c r="E76" t="s">
+        <v>22</v>
+      </c>
+      <c r="F76" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="77" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A77" s="17" t="s">
+        <v>114</v>
+      </c>
+      <c r="B77" s="18" t="s">
+        <v>116</v>
+      </c>
+      <c r="C77" s="18" t="s">
+        <v>117</v>
+      </c>
+      <c r="D77" s="18">
+        <v>75</v>
+      </c>
+      <c r="E77" t="s">
+        <v>102</v>
+      </c>
+      <c r="F77" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="78" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A78" t="s">
+        <v>10</v>
+      </c>
+      <c r="B78" t="s">
+        <v>14</v>
+      </c>
+      <c r="C78" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="D78">
+        <v>0.35</v>
+      </c>
+      <c r="E78" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="79" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A79" t="s">
+        <v>10</v>
+      </c>
+      <c r="B79" t="s">
+        <v>16</v>
+      </c>
+      <c r="C79" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="D79">
+        <v>5.68692529674572E-2</v>
+      </c>
+      <c r="E79" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="80" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A80" t="s">
+        <v>10</v>
+      </c>
+      <c r="B80" t="s">
+        <v>15</v>
+      </c>
+      <c r="C80" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="D80" s="3">
+        <v>0</v>
+      </c>
+      <c r="E80" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="81" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A81" t="s">
+        <v>10</v>
+      </c>
+      <c r="B81" t="s">
+        <v>9</v>
+      </c>
+      <c r="C81" s="3" t="s">
+        <v>107</v>
+      </c>
+      <c r="D81">
+        <v>4.2307926455512603E-2</v>
+      </c>
+      <c r="E81" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="82" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A82" t="s">
+        <v>10</v>
+      </c>
+      <c r="B82" t="s">
+        <v>87</v>
+      </c>
+      <c r="C82" s="14" t="s">
+        <v>11</v>
+      </c>
+      <c r="D82">
+        <v>0.57089503190107604</v>
+      </c>
+      <c r="E82" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="83" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A83" t="s">
+        <v>10</v>
+      </c>
+      <c r="B83" t="s">
+        <v>151</v>
+      </c>
+      <c r="C83" s="14" t="s">
+        <v>128</v>
+      </c>
+      <c r="D83">
+        <v>0.102978633031016</v>
+      </c>
+      <c r="E83" t="s">
+        <v>68</v>
+      </c>
+      <c r="F83" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="84" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A84" t="s">
+        <v>10</v>
+      </c>
+      <c r="B84" t="s">
+        <v>106</v>
+      </c>
+      <c r="C84" s="14" t="s">
+        <v>127</v>
+      </c>
+      <c r="D84" s="3">
+        <v>0.4</v>
+      </c>
+      <c r="E84" t="s">
+        <v>68</v>
+      </c>
+      <c r="F84" s="16">
+        <v>0.3</v>
+      </c>
+    </row>
+    <row r="85" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A85" t="s">
+        <v>10</v>
+      </c>
+      <c r="B85" t="s">
+        <v>140</v>
+      </c>
+      <c r="C85" s="14" t="s">
+        <v>141</v>
+      </c>
+      <c r="D85" s="3">
+        <v>0</v>
+      </c>
+      <c r="E85" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="86" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A86" t="s">
+        <v>10</v>
+      </c>
+      <c r="B86" t="s">
+        <v>154</v>
+      </c>
+      <c r="C86" s="14" t="s">
+        <v>152</v>
+      </c>
+      <c r="D86">
+        <v>2.86857836910057E-2</v>
+      </c>
+      <c r="E86" t="s">
+        <v>68</v>
+      </c>
+      <c r="F86" t="s">
+        <v>153</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7B05BFC5-2B20-4ACA-BF10-867F6673A613}">
+  <dimension ref="A1:F86"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="2" width="57.77734375" customWidth="1"/>
+    <col min="3" max="3" width="36" customWidth="1"/>
+    <col min="4" max="4" width="23" customWidth="1"/>
+    <col min="5" max="5" width="16.6640625" customWidth="1"/>
+    <col min="6" max="6" width="35.44140625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A2" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="D2" s="4">
+        <v>2000</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="F2" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A3" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="D3" s="4">
+        <v>16</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A4" s="4" t="s">
+        <v>163</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>164</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>165</v>
+      </c>
+      <c r="D4" s="4">
+        <v>2.5000000000000001E-3</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="F4" s="4" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A5" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="B5" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="C5" s="7" t="s">
+        <v>100</v>
+      </c>
+      <c r="D5" s="7">
+        <v>30</v>
+      </c>
+      <c r="E5" s="6" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A6" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="B6" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="C6" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="D6" s="6">
+        <v>40</v>
+      </c>
+      <c r="E6" s="6" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A7" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="B7" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="C7" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="D7" s="7">
+        <v>60</v>
+      </c>
+      <c r="E7" s="7" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A8" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="B8" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="C8" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="D8" s="7">
+        <v>60</v>
+      </c>
+      <c r="E8" s="7" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A9" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="B9" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="C9" s="8" t="s">
+        <v>57</v>
+      </c>
+      <c r="D9" s="8">
+        <v>60</v>
+      </c>
+      <c r="E9" s="8" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A10" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="B10" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="C10" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="D10" s="6">
+        <v>150</v>
+      </c>
+      <c r="E10" s="6" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A11" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="B11" s="7" t="s">
+        <v>64</v>
+      </c>
+      <c r="C11" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="D11" s="7">
+        <v>130</v>
+      </c>
+      <c r="E11" s="7" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A12" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="B12" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="C12" s="7" t="s">
+        <v>62</v>
+      </c>
+      <c r="D12" s="7">
+        <v>200</v>
+      </c>
+      <c r="E12" s="7" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A13" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="B13" s="7" t="s">
+        <v>66</v>
+      </c>
+      <c r="C13" s="7" t="s">
+        <v>63</v>
+      </c>
+      <c r="D13" s="7">
+        <v>70</v>
+      </c>
+      <c r="E13" s="7" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A14" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="B14" s="8" t="s">
+        <v>67</v>
+      </c>
+      <c r="C14" s="8" t="s">
+        <v>218</v>
+      </c>
+      <c r="D14" s="8">
+        <v>120</v>
+      </c>
+      <c r="E14" s="8" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A15" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="B15" s="7" t="s">
+        <v>83</v>
+      </c>
+      <c r="C15" s="7" t="s">
+        <v>82</v>
+      </c>
+      <c r="D15" s="7">
+        <v>110</v>
+      </c>
+      <c r="E15" s="8" t="s">
+        <v>85</v>
+      </c>
+      <c r="F15" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A16" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="B16" s="7" t="s">
+        <v>80</v>
+      </c>
+      <c r="C16" s="7" t="s">
+        <v>81</v>
+      </c>
+      <c r="D16" s="7">
+        <v>0.81</v>
+      </c>
+      <c r="E16" s="7" t="s">
+        <v>68</v>
+      </c>
+      <c r="F16" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A17" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="B17" s="7" t="s">
+        <v>111</v>
+      </c>
+      <c r="C17" s="7" t="s">
+        <v>109</v>
+      </c>
+      <c r="D17" s="7">
+        <v>0</v>
+      </c>
+      <c r="E17" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="F17" s="7" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A18" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="B18" s="7" t="s">
+        <v>119</v>
+      </c>
+      <c r="C18" s="7" t="s">
+        <v>121</v>
+      </c>
+      <c r="D18" s="7">
+        <v>0.3</v>
+      </c>
+      <c r="E18" s="7" t="s">
+        <v>68</v>
+      </c>
+      <c r="F18" s="7" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A19" s="15" t="s">
+        <v>17</v>
+      </c>
+      <c r="B19" s="15" t="s">
+        <v>130</v>
+      </c>
+      <c r="C19" s="15" t="s">
+        <v>101</v>
+      </c>
+      <c r="D19" s="15">
+        <v>30</v>
+      </c>
+      <c r="E19" s="15" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A20" s="15" t="s">
+        <v>17</v>
+      </c>
+      <c r="B20" s="15" t="s">
+        <v>103</v>
+      </c>
+      <c r="C20" s="15" t="s">
+        <v>108</v>
+      </c>
+      <c r="D20" s="15">
+        <v>30</v>
+      </c>
+      <c r="E20" s="15" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A21" s="15" t="s">
+        <v>17</v>
+      </c>
+      <c r="B21" s="15" t="s">
+        <v>104</v>
+      </c>
+      <c r="C21" s="15" t="s">
+        <v>105</v>
+      </c>
+      <c r="D21" s="15">
+        <v>8</v>
+      </c>
+      <c r="E21" s="15" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A22" s="15" t="s">
+        <v>17</v>
+      </c>
+      <c r="B22" s="15" t="s">
+        <v>129</v>
+      </c>
+      <c r="C22" s="15" t="s">
+        <v>131</v>
+      </c>
+      <c r="D22" s="15">
+        <v>2.2999999999999998</v>
+      </c>
+      <c r="E22" s="15" t="s">
+        <v>132</v>
+      </c>
+      <c r="F22" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A23" s="15" t="s">
+        <v>17</v>
+      </c>
+      <c r="B23" s="15" t="s">
+        <v>134</v>
+      </c>
+      <c r="C23" s="15" t="s">
+        <v>137</v>
+      </c>
+      <c r="D23" s="15">
+        <v>1.25</v>
+      </c>
+      <c r="E23" s="15"/>
+      <c r="F23" s="15" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A24" s="15" t="s">
+        <v>17</v>
+      </c>
+      <c r="B24" s="15" t="s">
+        <v>135</v>
+      </c>
+      <c r="C24" s="15" t="s">
+        <v>138</v>
+      </c>
+      <c r="D24" s="15">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="E24" s="15"/>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A25" s="15" t="s">
+        <v>17</v>
+      </c>
+      <c r="B25" s="15" t="s">
+        <v>136</v>
+      </c>
+      <c r="C25" s="15" t="s">
+        <v>139</v>
+      </c>
+      <c r="D25" s="15">
+        <v>1.08</v>
+      </c>
+      <c r="E25" s="15"/>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A26" s="15" t="s">
+        <v>17</v>
+      </c>
+      <c r="B26" s="15" t="s">
+        <v>179</v>
+      </c>
+      <c r="C26" s="15" t="s">
+        <v>180</v>
+      </c>
+      <c r="D26" s="15">
+        <v>0.3</v>
+      </c>
+      <c r="E26" s="15" t="s">
+        <v>68</v>
+      </c>
+      <c r="F26" s="15" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A27" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="B27" s="10" t="s">
+        <v>99</v>
+      </c>
+      <c r="C27" s="10" t="s">
+        <v>181</v>
+      </c>
+      <c r="D27" s="10">
+        <v>0.6</v>
+      </c>
+      <c r="E27" s="10" t="s">
+        <v>68</v>
+      </c>
+      <c r="F27" s="9" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A28" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="B28" s="5" t="s">
+        <v>69</v>
+      </c>
+      <c r="C28" s="5" t="s">
+        <v>223</v>
+      </c>
+      <c r="D28" s="5">
+        <v>11.8</v>
+      </c>
+      <c r="E28" s="5" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A29" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="B29" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="C29" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="D29" s="5">
+        <v>11.8</v>
+      </c>
+      <c r="E29" s="5" t="s">
+        <v>146</v>
+      </c>
+      <c r="F29" s="5"/>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A30" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="B30" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="C30" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="D30" s="5">
+        <v>11.8</v>
+      </c>
+      <c r="E30" s="5" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A31" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="B31" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="C31" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="D31" s="5">
+        <v>11.8</v>
+      </c>
+      <c r="E31" s="5" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A32" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="B32" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="C32" s="5" t="s">
+        <v>224</v>
+      </c>
+      <c r="D32" s="5">
+        <v>13.2</v>
+      </c>
+      <c r="E32" s="5" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A33" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="B33" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="C33" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="D33" s="5">
+        <v>13.2</v>
+      </c>
+      <c r="E33" s="5" t="s">
+        <v>146</v>
+      </c>
+      <c r="F33" s="5" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A34" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="B34" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="C34" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="D34" s="5">
+        <v>13.2</v>
+      </c>
+      <c r="E34" s="5" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A35" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="B35" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="C35" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="D35" s="5">
+        <v>13.2</v>
+      </c>
+      <c r="E35" s="5" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A36" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="B36" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="C36" s="5" t="s">
+        <v>225</v>
+      </c>
+      <c r="D36" s="5">
+        <v>35.4</v>
+      </c>
+      <c r="E36" s="5" t="s">
+        <v>146</v>
+      </c>
+      <c r="F36" s="5"/>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A37" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="B37" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="C37" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="D37" s="5">
+        <v>35.4</v>
+      </c>
+      <c r="E37" s="5" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A38" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="B38" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="C38" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="D38" s="5">
+        <v>35.4</v>
+      </c>
+      <c r="E38" s="5" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A39" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="B39" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="C39" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D39" s="5">
+        <v>35.4</v>
+      </c>
+      <c r="E39" s="5" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A40" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="B40" s="5" t="s">
+        <v>90</v>
+      </c>
+      <c r="C40" s="5" t="s">
+        <v>93</v>
+      </c>
+      <c r="D40" s="5">
+        <v>0.3</v>
+      </c>
+      <c r="E40" s="5"/>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A41" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="B41" s="5" t="s">
+        <v>90</v>
+      </c>
+      <c r="C41" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="D41" s="5">
+        <v>0.3</v>
+      </c>
+      <c r="E41" s="5"/>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A42" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="B42" s="5" t="s">
+        <v>90</v>
+      </c>
+      <c r="C42" s="5" t="s">
+        <v>95</v>
+      </c>
+      <c r="D42" s="5">
+        <v>0.3</v>
+      </c>
+      <c r="E42" s="5"/>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A43" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="B43" s="5" t="s">
+        <v>90</v>
+      </c>
+      <c r="C43" s="5" t="s">
+        <v>96</v>
+      </c>
+      <c r="D43" s="5">
+        <v>0.3</v>
+      </c>
+      <c r="E43" s="5"/>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A44" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="B44" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="C44" s="5" t="s">
+        <v>226</v>
+      </c>
+      <c r="D44" s="5">
+        <v>11.4</v>
+      </c>
+      <c r="E44" s="5"/>
+      <c r="F44" s="5" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A45" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="B45" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="C45" s="5" t="s">
+        <v>219</v>
+      </c>
+      <c r="D45" s="5">
+        <v>11.4</v>
+      </c>
+      <c r="E45" s="5"/>
+      <c r="F45" s="5" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A46" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="B46" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="C46" s="5" t="s">
+        <v>220</v>
+      </c>
+      <c r="D46" s="5">
+        <v>11.4</v>
+      </c>
+      <c r="E46" s="5"/>
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A47" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="B47" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="C47" s="5" t="s">
+        <v>221</v>
+      </c>
+      <c r="D47" s="5">
+        <v>11.4</v>
+      </c>
+      <c r="E47" s="5"/>
+    </row>
+    <row r="48" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A48" s="11" t="s">
+        <v>6</v>
+      </c>
+      <c r="B48" s="11" t="s">
+        <v>174</v>
+      </c>
+      <c r="C48" s="12" t="s">
+        <v>175</v>
+      </c>
+      <c r="D48" s="13">
+        <v>700</v>
+      </c>
+      <c r="E48" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A49" s="11" t="s">
+        <v>6</v>
+      </c>
+      <c r="B49" s="11" t="s">
+        <v>39</v>
+      </c>
+      <c r="C49" s="12" t="s">
+        <v>41</v>
+      </c>
+      <c r="D49" s="13">
+        <v>0.13500000000000001</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A50" s="11" t="s">
+        <v>6</v>
+      </c>
+      <c r="B50" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="C50" s="12" t="s">
+        <v>42</v>
+      </c>
+      <c r="D50" s="13">
+        <v>0.23</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A51" s="11" t="s">
+        <v>6</v>
+      </c>
+      <c r="B51" s="13" t="s">
+        <v>70</v>
+      </c>
+      <c r="C51" s="12" t="s">
+        <v>76</v>
+      </c>
+      <c r="D51" s="13">
+        <v>2018.3</v>
+      </c>
+      <c r="E51" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A52" s="11" t="s">
+        <v>6</v>
+      </c>
+      <c r="B52" s="13" t="s">
+        <v>71</v>
+      </c>
+      <c r="C52" s="12" t="s">
+        <v>78</v>
+      </c>
+      <c r="D52" s="13">
+        <v>2022.15</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A53" s="11" t="s">
+        <v>6</v>
+      </c>
+      <c r="B53" s="13" t="s">
+        <v>88</v>
+      </c>
+      <c r="C53" s="12" t="s">
+        <v>89</v>
+      </c>
+      <c r="D53" s="13">
+        <v>2011</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A54" s="11" t="s">
+        <v>6</v>
+      </c>
+      <c r="B54" s="13" t="s">
+        <v>122</v>
+      </c>
+      <c r="C54" s="12" t="s">
+        <v>124</v>
+      </c>
+      <c r="D54" s="13">
+        <v>150</v>
+      </c>
+      <c r="E54" s="13" t="s">
+        <v>102</v>
+      </c>
+      <c r="F54" s="13" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A55" s="11" t="s">
+        <v>6</v>
+      </c>
+      <c r="B55" s="13" t="s">
+        <v>176</v>
+      </c>
+      <c r="C55" s="12" t="s">
+        <v>178</v>
+      </c>
+      <c r="D55" s="13">
+        <v>35000</v>
+      </c>
+      <c r="E55" s="13" t="s">
+        <v>22</v>
+      </c>
+      <c r="F55" s="13"/>
+    </row>
+    <row r="56" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A56" s="11" t="s">
+        <v>6</v>
+      </c>
+      <c r="B56" s="13" t="s">
+        <v>123</v>
+      </c>
+      <c r="C56" s="12" t="s">
+        <v>125</v>
+      </c>
+      <c r="D56" s="13">
+        <v>2027</v>
+      </c>
+      <c r="E56" s="13" t="s">
+        <v>126</v>
+      </c>
+      <c r="F56" s="13" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="57" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A57" s="11" t="s">
+        <v>6</v>
+      </c>
+      <c r="B57" s="13" t="s">
+        <v>203</v>
+      </c>
+      <c r="C57" s="12" t="s">
+        <v>205</v>
+      </c>
+      <c r="D57" s="13">
+        <v>2028.5</v>
+      </c>
+      <c r="E57" s="13"/>
+      <c r="F57" s="13"/>
+    </row>
+    <row r="58" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A58" s="11" t="s">
+        <v>6</v>
+      </c>
+      <c r="B58" s="13" t="s">
+        <v>204</v>
+      </c>
+      <c r="C58" s="12" t="s">
+        <v>209</v>
+      </c>
+      <c r="D58" s="13">
+        <v>120</v>
+      </c>
+      <c r="E58" s="13" t="s">
+        <v>208</v>
+      </c>
+      <c r="F58" s="13"/>
+    </row>
+    <row r="59" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A59" s="11" t="s">
+        <v>6</v>
+      </c>
+      <c r="B59" s="13" t="s">
+        <v>206</v>
+      </c>
+      <c r="C59" s="12" t="s">
+        <v>207</v>
+      </c>
+      <c r="D59" s="13">
+        <v>45000</v>
+      </c>
+      <c r="E59" s="13" t="s">
+        <v>22</v>
+      </c>
+      <c r="F59" s="13"/>
+    </row>
+    <row r="60" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A60" s="11" t="s">
+        <v>6</v>
+      </c>
+      <c r="B60" s="13" t="s">
+        <v>97</v>
+      </c>
+      <c r="C60" s="12" t="s">
+        <v>98</v>
+      </c>
+      <c r="D60" s="13">
+        <v>2015.3</v>
+      </c>
+    </row>
+    <row r="61" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A61" s="11" t="s">
+        <v>6</v>
+      </c>
+      <c r="B61" s="13" t="s">
+        <v>72</v>
+      </c>
+      <c r="C61" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="D61" s="13">
+        <v>2024.3</v>
+      </c>
+      <c r="E61" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A62" s="11" t="s">
+        <v>6</v>
+      </c>
+      <c r="B62" s="13" t="s">
+        <v>79</v>
+      </c>
+      <c r="C62" s="12" t="s">
+        <v>77</v>
+      </c>
+      <c r="D62" s="13">
+        <v>2040</v>
+      </c>
+    </row>
+    <row r="63" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A63" s="11" t="s">
+        <v>6</v>
+      </c>
+      <c r="B63" s="13" t="s">
+        <v>91</v>
+      </c>
+      <c r="C63" s="12" t="s">
+        <v>92</v>
+      </c>
+      <c r="D63" s="13">
+        <v>2040</v>
+      </c>
+    </row>
+    <row r="64" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A64" s="11" t="s">
+        <v>6</v>
+      </c>
+      <c r="B64" s="13" t="s">
+        <v>142</v>
+      </c>
+      <c r="C64" s="13" t="s">
+        <v>144</v>
+      </c>
+      <c r="D64" s="13">
+        <v>0.8</v>
+      </c>
+      <c r="E64" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="65" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A65" s="11" t="s">
+        <v>6</v>
+      </c>
+      <c r="B65" s="13" t="s">
+        <v>197</v>
+      </c>
+      <c r="C65" s="13" t="s">
+        <v>193</v>
+      </c>
+      <c r="D65" s="13">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="66" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A66" s="11" t="s">
+        <v>6</v>
+      </c>
+      <c r="B66" s="13" t="s">
+        <v>170</v>
+      </c>
+      <c r="C66" s="13" t="s">
+        <v>194</v>
+      </c>
+      <c r="D66" s="13">
+        <v>63.5</v>
+      </c>
+      <c r="E66" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A67" s="11" t="s">
+        <v>6</v>
+      </c>
+      <c r="B67" s="13" t="s">
+        <v>171</v>
+      </c>
+      <c r="C67" s="13" t="s">
+        <v>195</v>
+      </c>
+      <c r="D67" s="13">
+        <v>200</v>
+      </c>
+      <c r="E67" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="68" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A68" s="11" t="s">
+        <v>6</v>
+      </c>
+      <c r="B68" s="13" t="s">
+        <v>172</v>
+      </c>
+      <c r="C68" s="13" t="s">
+        <v>196</v>
+      </c>
+      <c r="D68" s="13">
+        <v>400</v>
+      </c>
+      <c r="E68" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="69" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A69" s="11" t="s">
+        <v>6</v>
+      </c>
+      <c r="B69" s="13" t="s">
+        <v>185</v>
+      </c>
+      <c r="C69" s="13" t="s">
+        <v>187</v>
+      </c>
+      <c r="D69" s="13">
+        <v>2026.5</v>
+      </c>
+    </row>
+    <row r="70" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A70" s="11" t="s">
+        <v>6</v>
+      </c>
+      <c r="B70" s="13" t="s">
+        <v>186</v>
+      </c>
+      <c r="C70" s="13" t="s">
+        <v>188</v>
+      </c>
+      <c r="D70" s="13">
+        <v>1.6</v>
+      </c>
+    </row>
+    <row r="71" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A71" s="11" t="s">
+        <v>6</v>
+      </c>
+      <c r="B71" s="13" t="s">
+        <v>190</v>
+      </c>
+      <c r="C71" s="13" t="s">
+        <v>189</v>
+      </c>
+      <c r="D71" s="13">
+        <v>2031</v>
+      </c>
+    </row>
+    <row r="72" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A72" s="11" t="s">
+        <v>6</v>
+      </c>
+      <c r="B72" s="13" t="s">
+        <v>191</v>
+      </c>
+      <c r="C72" s="13" t="s">
+        <v>192</v>
+      </c>
+      <c r="D72" s="13">
+        <v>2041</v>
+      </c>
+    </row>
+    <row r="73" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A73" s="11" t="s">
+        <v>6</v>
+      </c>
+      <c r="B73" s="13" t="s">
+        <v>129</v>
+      </c>
+      <c r="C73" s="13" t="s">
+        <v>198</v>
+      </c>
+      <c r="D73" s="13">
+        <v>2032</v>
+      </c>
+    </row>
+    <row r="74" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A74" s="11" t="s">
+        <v>6</v>
+      </c>
+      <c r="B74" s="13" t="s">
+        <v>129</v>
+      </c>
+      <c r="C74" s="13" t="s">
+        <v>199</v>
+      </c>
+      <c r="D74" s="13">
+        <v>2.8</v>
       </c>
     </row>
     <row r="75" spans="1:6" x14ac:dyDescent="0.3">

</xml_diff>